<commit_message>
feat(F-NAR-019): ATOM-DIF.PAR.002-03 Nina laisse le temps à Aniss
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.PAR.002-03.xlsx
+++ b/stories/arbres/ATOM-DIF.PAR.002-03.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le chat bleu de Nina</t>
+          <t>Nina laisse le temps à Aniss</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>salon</t>
+          <t>maison, salon, goûter, plateau, cacao, dessin, crayon bleu, verre d'eau, table</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nino, Nina, papa, maman</t>
+          <t>Nina, Aniss, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nina veut raconter son chat bleu. Nino a envie de finir. Il pose ses mains. Nina dit le mot. Plus tard, elle demande de l'eau, tout doucement.</t>
+          <t>Le plateau du goûter pose une ombre. Près du cacao, un éclat de plateau brille. Nina veut aider Aniss, maintenant. Le mot du dessin reste dedans. Nina ouvre la bouche trop vite. Sourire parti, poitrine, papa accroupi. Elle referme la bouche, attend. Merci vécu. Verre trop vite. Elle s'arrête, lit l'éclat. Un éclat de plateau tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La lampe du salon fait une lune ronde sur le tapis. Un coussin a encore le creux de quelqu'un. Ça sent le cacao, un peu sucré. La petite horloge avance tout doucement. Le goûter est prêt. Compote et cacao, d'accord ? Je m'assois sur le tapis. Il est doux, ce tapis. En ce moment, Nino est assis près de la table basse. Ses chaussettes glissent un peu sur le tapis. Tu veux la petite cuillère bleue ? Oui, maman. La cuillère tinte contre le bol. Nina tient un dessin. Le papier est un peu plié. Le... Nina cherche le mot. Nino voit le crayon bleu. Il a envie de finir. On laisse le temps, Nino. On attend la fin de la phrase. Nino pose ses mains sur ses genoux. Il attend. L'horloge fait un tout petit tic. Le chat bleu. J'aime le chat. Bravo, Nino. Tu as laissé le temps. Nina pose le dessin contre le bol. Le cacao fume encore un peu. Je... je... Nina veut un verre. Nino attend encore. Il regarde la lune sur le tapis. Je veux de l'eau. Voici le verre, Nina. Tu as fini ta phrase, toute seule. Nino, tu as écouté jusqu'au bout ? Oui, papa. On laisse le temps. Nino croque une cuillère de compote. C'est doux, ça colle un peu. Le chat, il a... Nino attend la fin. Il a des moustaches. Des moustaches, oui. Vous parlez l'un après l'autre. Vous avez fini votre goûter ? Presque, maman. Nina montre encore le chat bleu. Nino a attendu la fin de la phrase. Le cacao n'est plus tout chaud. On range le dessin après, d'accord ? D'accord. Nino attend que Nina finisse. Puis il hoche la tête.</t>
+          <t>Le plateau du goûter pose une ombre chaude sur la table. Ça sent le cacao, un peu sucré. Ça sent bon, papa. Tu le sens, le cacao, Nina ? Oui, papa. La vapeur danse au-dessus des tasses. Elle monte, maman. Le cacao fume ? Oui. Le goûter est prêt. Cacao et compote, d'accord ? Oui, maman. Un crayon bleu roule vers le bord. Il roule, papa. Tu le rattrapes, Nina ? Oui. La cuillère tinte contre le bol. Elle chante, maman. Tu l'entends, la cuillère ? Oui. Près du cacao, un éclat de plateau brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Une poussière danse au-dessus du plateau. Elle vole, maman. Au-dessus du cacao ? Oui, au-dessus. Aniss pose un dessin sur la table. Le papier est un peu plié. C'est ton dessin, Aniss ? Aniss serre le crayon. Le crayon laisse une trace bleue. C'est bleu, papa. Comme le ciel ? Oui, comme le ciel. En ce moment, Nina se penche vers la feuille. Je veux aider, maintenant ! Je connais le mot. Tu vois Aniss, Nina ? Oui, papa. Aniss ouvre la bouche. Le mot reste dedans. Ses épaules montent un peu. Le chat ! Nina ouvre la bouche trop vite. Les mots montent. Aniss baisse les yeux. Oh. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Il cherche, Nina ? Oui, papa. Tes lèvres sont ouvertes, Nina ? Un peu, maman. L'éclat de plateau tremble, puis tient. Aniss tient le dessin contre lui. Il ne dit pas le mot, papa. Papa s'accroupit à la même hauteur. Nina regarde papa.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La lampe du salon fait une lune ronde sur le tapis. Un coussin a encore le creux de quelqu'un. Ça sent le cacao, un peu sucré. La petite horloge avance tout doucement. Le goûter est prêt. Compote et cacao, d'accord ? Je m'assois sur le tapis. Il est doux, ce tapis. En ce moment, Nino est assis près de la table basse. Ses chaussettes glissent un peu sur le tapis. Tu veux la petite cuillère bleue ? Oui, maman. La cuillère tinte contre le bol. Nina tient un dessin. Le papier est un peu plié. Le... Nina cherche le mot. Nino voit le crayon bleu. Il a envie de finir. On laisse le temps, Nino. On attend la fin de la phrase. Nino pose ses mains sur ses genoux. Il attend. L'horloge fait un tout petit tic. Le chat bleu. J'aime le chat. Bravo, Nino. Tu as laissé le temps. Nina pose le dessin contre le bol. Le cacao fume encore un peu. Je... je... Nina veut un verre. Nino attend encore. Il regarde la lune sur le tapis. Je veux de l'eau. Voici le verre, Nina. Tu as fini ta phrase, toute seule. Nino, tu as écouté jusqu'au bout ? Oui, papa. On laisse le temps. Nino croque une cuillère de compote. C'est doux, ça colle un peu. Le chat, il a... Nino attend la fin. Il a des moustaches. Des moustaches, oui. Vous parlez l'un après l'autre. Vous avez fini votre goûter ? Presque, maman. Nina montre encore le chat bleu. Nino a attendu la fin de la phrase. Le cacao n'est plus tout chaud. On range le dessin après, d'accord ? D'accord. Nino attend que Nina finisse. Puis il hoche la tête.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le plateau du goûter pose une ombre chaude sur la table. Ça sent le cacao, un peu sucré. Ça sent bon, papa. Tu le sens, le cacao, Nina ? Oui, papa. La vapeur danse au-dessus des tasses. Elle monte, maman. Le cacao fume ? Oui. Le goûter est prêt. Cacao et compote, d'accord ? Oui, maman. Un crayon bleu roule vers le bord. Il roule, papa. Tu le rattrapes, Nina ? Oui. La cuillère tinte contre le bol. Elle chante, maman. Tu l'entends, la cuillère ? Oui. Près du cacao, un &lt;emphasis level="moderate"&gt;éclat de plateau&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Une poussière danse au-dessus du plateau. Elle vole, maman. Au-dessus du cacao ? Oui, au-dessus. Aniss pose un dessin sur la table. Le papier est un peu plié. C'est ton dessin, Aniss ? Aniss serre le crayon. Le crayon laisse une trace bleue. C'est bleu, papa. Comme le ciel ? Oui, comme le ciel. En ce moment, Nina se penche vers la feuille. Je veux aider, maintenant ! Je connais le mot. Tu vois Aniss, Nina ? Oui, papa. Aniss ouvre la bouche. Le mot reste dedans. Ses épaules montent un peu. Le chat ! Nina ouvre la bouche trop vite. Les mots montent. Aniss baisse les yeux. Oh. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Il cherche, Nina ? Oui, papa. Tes lèvres sont ouvertes, Nina ? Un peu, maman. L'éclat de plateau tremble, puis tient. Aniss tient le dessin contre lui. Il ne dit pas le mot, papa. Papa s'accroupit à la même hauteur. Nina regarde papa.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Céleste et Sami sont dans le salon. Maman pose le goûter. Papa s'assoit sur le tapis. Sami veut raconter son dessin. Il cherche les mots. Il dit : le.. le.. Céleste a envie de finir. Papa dit : on laisse le temps. Céleste attend. Elle pose ses &lt;emphasis&gt;main&lt;/emphasis&gt;s sur ses genoux. Sami dit : le chat bleu. Parce qu'on a laissé le temps, Sami a fini sa phrase. Céleste sourit. Elle dit : j'aime le chat. Plus tard, Sami veut un verre. Il dit : je.. je.. Céleste attend encore. Elle laisse le temps. Sami dit : je veux de l'eau. Maman tend le verre. Céleste n'a pas parlé à sa place. Elle a attendu la fin de la phrase. [pause]</t>
+          <t>Le plateau du goûter pose une ombre chaude sur la table. Ça sent le cacao, un peu sucré. Ça sent bon, papa. Tu le sens, le cacao, Nina ? Oui, papa. La vapeur danse au-dessus des tasses. Elle monte, maman. Le cacao fume ? Oui. Le goûter est prêt. Cacao et compote, d'accord ? Oui, maman. Un crayon bleu roule vers le bord. Il roule, papa. Tu le rattrapes, Nina ? Oui. La cuillère tinte contre le bol. Elle chante, maman. Tu l'entends, la cuillère ? Oui. Près du cacao, un &lt;emphasis&gt;éclat de plateau&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Une poussière danse au-dessus du plateau. Elle vole, maman. Au-dessus du cacao ? Oui, au-dessus. Aniss pose un dessin sur la table. Le papier est un peu plié. C'est ton dessin, Aniss ? Aniss serre le crayon. Le crayon laisse une trace bleue. C'est bleu, papa. Comme le ciel ? Oui, comme le ciel. En ce moment, Nina se penche vers la feuille. Je veux aider, maintenant ! Je connais le mot. Tu vois Aniss, Nina ? Oui, papa. Aniss ouvre la bouche. Le mot reste dedans. Ses épaules montent un peu. Le chat ! Nina ouvre la bouche trop vite. Les mots montent. Aniss baisse les yeux. Oh. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Il cherche, Nina ? Oui, papa. Tes lèvres sont ouvertes, Nina ? Un peu, maman. L'éclat de plateau tremble, puis tient. Aniss tient le dessin contre lui. Il ne dit pas le mot, papa. Papa s'accroupit à la même hauteur. Nina regarde papa. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de plateau</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,65 +1321,74 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_aider_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La lampe du salon fait une lune ronde sur le tapis.
-narrateur|Un coussin a encore le creux de quelqu'un.
+          <t>narrateur|Le plateau du goûter pose une ombre chaude sur la table.
 narrateur|Ça sent le cacao, un peu sucré.
-narrateur|La petite horloge avance tout doucement.
+enfant-f|Ça sent bon, papa.
+papa|Tu le sens, le cacao, Nina ?
+enfant-f|Oui, papa.
+narrateur|La vapeur danse au-dessus des tasses.
+enfant-f|Elle monte, maman.
+maman|Le cacao fume ?
+enfant-f|Oui.
 maman|Le goûter est prêt.
-maman|Compote et cacao, d'accord ?
-papa|Je m'assois sur le tapis.
-papa|Il est doux, ce tapis.
-narrateur|En ce moment, Nino est assis près de la table basse.
-narrateur|Ses chaussettes glissent un peu sur le tapis.
-maman|Tu veux la petite cuillère bleue ?
-enfant-m|Oui, maman.
+maman|Cacao et compote, d'accord ?
+enfant-f|Oui, maman.
+narrateur|Un crayon bleu roule vers le bord.
+enfant-f|Il roule, papa.
+papa|Tu le rattrapes, Nina ?
+enfant-f|Oui.
 narrateur|La cuillère tinte contre le bol.
-narrateur|Nina tient un dessin.
+enfant-f|Elle chante, maman.
+maman|Tu l'entends, la cuillère ?
+enfant-f|Oui.
+narrateur|Près du cacao, un éclat de plateau brille.
+enfant-f|Il brille, papa.
+papa|Tu le vois, le petit point ?
+enfant-f|Oui, un petit point.
+narrateur|Une poussière danse au-dessus du plateau.
+enfant-f|Elle vole, maman.
+maman|Au-dessus du cacao ?
+enfant-f|Oui, au-dessus.
+narrateur|Aniss pose un dessin sur la table.
 narrateur|Le papier est un peu plié.
-copine|Le...
-narrateur|Nina cherche le mot.
-narrateur|Nino voit le crayon bleu.
-narrateur|Il a envie de finir.
-papa|On laisse le temps, Nino.
-papa|On attend la fin de la phrase.
-narrateur|Nino pose ses mains sur ses genoux.
-narrateur|Il attend.
-narrateur|L'horloge fait un tout petit tic.
-copine|Le chat bleu.
-enfant-m|J'aime le chat.
-maman|Bravo, Nino.
-maman|Tu as laissé le temps.
-narrateur|Nina pose le dessin contre le bol.
-narrateur|Le cacao fume encore un peu.
-copine|Je... je...
-narrateur|Nina veut un verre.
-narrateur|Nino attend encore.
-narrateur|Il regarde la lune sur le tapis.
-copine|Je veux de l'eau.
-maman|Voici le verre, Nina.
-maman|Tu as fini ta phrase, toute seule.
-papa|Nino, tu as écouté jusqu'au bout ?
-enfant-m|Oui, papa.
-papa|On laisse le temps.
-narrateur|Nino croque une cuillère de compote.
-narrateur|C'est doux, ça colle un peu.
-copine|Le chat, il a...
-narrateur|Nino attend la fin.
-copine|Il a des moustaches.
-enfant-m|Des moustaches, oui.
-maman|Vous parlez l'un après l'autre.
-maman|Vous avez fini votre goûter ?
-enfant-m|Presque, maman.
-narrateur|Nina montre encore le chat bleu.
-narrateur|Nino a attendu la fin de la phrase.
-narrateur|Le cacao n'est plus tout chaud.
-papa|On range le dessin après, d'accord ?
-copine|D'accord.
-narrateur|Nino attend que Nina finisse.
-narrateur|Puis il hoche la tête.</t>
+enfant-f|C'est ton dessin, Aniss ?
+narrateur|Aniss serre le crayon.
+narrateur|Le crayon laisse une trace bleue.
+enfant-f|C'est bleu, papa.
+papa|Comme le ciel ?
+enfant-f|Oui, comme le ciel.
+narrateur|En ce moment, Nina se penche vers la feuille.
+enfant-f|Je veux aider, maintenant !
+enfant-f|Je connais le mot.
+papa|Tu vois Aniss, Nina ?
+enfant-f|Oui, papa.
+narrateur|Aniss ouvre la bouche.
+narrateur|Le mot reste dedans.
+narrateur|Ses épaules montent un peu.
+enfant-f|Le chat !
+narrateur|Nina ouvre la bouche trop vite.
+narrateur|Les mots montent.
+narrateur|Aniss baisse les yeux.
+enfant-f|Oh.
+narrateur|Le sourire de Nina disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+papa|Il cherche, Nina ?
+enfant-f|Oui, papa.
+maman|Tes lèvres sont ouvertes, Nina ?
+enfant-f|Un peu, maman.
+narrateur|L'éclat de plateau tremble, puis tient.
+narrateur|Aniss tient le dessin contre lui.
+enfant-f|Il ne dit pas le mot, papa.
+narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Nina regarde papa.</t>
         </is>
       </c>
     </row>
@@ -1406,17 +1415,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Nina cherche ses mots. Que fait Nino ?</t>
+          <t>Aniss cherche ses mots. Que fait Nina ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nina cherche ses mots. Que fait Nino ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Aniss cherche ses mots. Que fait &lt;emphasis level="moderate"&gt;Nina&lt;/emphasis&gt; ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Sami cherche ses mots. Que fait Céleste ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Aniss cherche ses mots. Que fait &lt;emphasis&gt;Nina&lt;/emphasis&gt; ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1441,7 +1450,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>On laisse le temps. On attend la fin. Que fait Céleste ?</t>
+          <t>On laisse le temps. On attend la fin. Que fait Nina ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1479,7 +1488,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1490,7 +1499,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1505,34 +1514,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Nina</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1547,23 +1560,23 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=aniss_cherche_ses_mots_que_fait_nina; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Nina cherche ses mots.
-narrateur|Que fait Nino ?</t>
+          <t>narrateur|Aniss cherche ses mots.
+narrateur|Que fait Nina ?</t>
         </is>
       </c>
     </row>
@@ -1590,17 +1603,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nino a laissé le temps. Nina a fini sa phrase. On attend la fin de la phrase. Bravo, Nino. J'ai laissé le temps.</t>
+          <t>Nina veut le mot, tout de suite. Je le dis, maintenant ! Elle avance trop vite vers Aniss. Les mots se bousculent dans sa bouche. Aniss baisse les yeux. Il serre le dessin contre lui. Oh. Le sourire ne revient pas. Nina ouvre la bouche. Puis elle la referme. Personne ne parle. Elle observe le dessin, un instant. Elle écoute la vapeur du cacao. Tu veux le chat avec Aniss ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose les mains, puis on reste. D'accord. Nina reste un moment, les mains ouvertes. Elle attend. Aniss souffle. Le chat bleu. J'aime le chat. Aniss pose le dessin contre le plateau. Merci, Nina. Papa a vu les deux, au salon. Le papier est tiède, sous les doigts. Il est chaud. Le chat bleu tient, un peu de travers. Le chat. Il a une oreille, là ? Oui, là. Nina glisse la main près du dessin. Le papier est doux, contre la peau. Tes mains sont au chaud, Nina ? Un peu, maman. Aniss s'assoit, puis se relève. Oui. On le pose au bord ? Le plateau va jusqu'à la table. Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nino a laissé le temps. Nina a fini sa phrase. On attend la fin de la phrase. Bravo, Nino. J'ai laissé le temps.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina veut le mot, tout de suite. Je le dis, maintenant ! Elle avance trop vite vers Aniss. Les mots se bousculent dans sa bouche. Aniss baisse les yeux. Il serre le dessin contre lui. Oh. Le sourire ne revient pas. Nina ouvre la bouche. Puis elle la referme. Personne ne parle. Elle observe le dessin, un instant. Elle écoute la vapeur du cacao. Tu veux le &lt;emphasis level="moderate"&gt;chat&lt;/emphasis&gt; avec Aniss ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose les mains, puis on reste. D'accord. Nina reste un moment, les mains ouvertes. Elle attend. Aniss souffle. Le chat bleu. J'aime le chat. Aniss pose le dessin contre le plateau. Merci, Nina. Papa a vu les deux, au salon. Le papier est tiède, sous les doigts. Il est chaud. Le chat bleu tient, un peu de travers. Le chat. Il a une oreille, là ? Oui, là. Nina glisse la main près du dessin. Le papier est doux, contre la peau. Tes mains sont au chaud, Nina ? Un peu, maman. Aniss s'assoit, puis se relève. Oui. On le pose au bord ? Le plateau va jusqu'à la table. Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Céleste a laissé le temps. Sami a fini sa phrase. Papa et maman étaient là. [pause]</t>
+          <t>Nina veut le mot, tout de suite. Je le dis, maintenant ! Elle avance trop vite vers Aniss. Les mots se bousculent dans sa bouche. Aniss baisse les yeux. Il serre le dessin contre lui. Oh. Le sourire ne revient pas. Nina ouvre la bouche. Puis elle la referme. Personne ne parle. Elle observe le dessin, un instant. Elle écoute la vapeur du cacao. Tu veux le &lt;emphasis&gt;chat&lt;/emphasis&gt; avec Aniss ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose les mains, puis on reste. D'accord. Nina reste un moment, les mains ouvertes. Elle attend. Aniss souffle. Le chat bleu. J'aime le chat. Aniss pose le dessin contre le plateau. Merci, Nina. Papa a vu les deux, au salon. Le papier est tiède, sous les doigts. Il est chaud. Le chat bleu tient, un peu de travers. Le chat. Il a une oreille, là ? Oui, là. Nina glisse la main près du dessin. Le papier est doux, contre la peau. Tes mains sont au chaud, Nina ? Un peu, maman. Aniss s'assoit, puis se relève. Oui. On le pose au bord ? Le plateau va jusqu'à la table. Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1647,7 +1660,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1655,10 +1668,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1679,28 +1692,32 @@
       <c r="AG4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr">
+        <is>
+          <t>chat</t>
+        </is>
+      </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1709,10 +1726,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1725,16 +1742,52 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_ouvre_referme_attend; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nino a laissé le temps.
-narrateur|Nina a fini sa phrase.
-papa|On attend la fin de la phrase.
-maman|Bravo, Nino.
-enfant-m|J'ai laissé le temps.</t>
+          <t>narrateur|Nina veut le mot, tout de suite.
+enfant-f|Je le dis, maintenant !
+narrateur|Elle avance trop vite vers Aniss.
+narrateur|Les mots se bousculent dans sa bouche.
+narrateur|Aniss baisse les yeux.
+narrateur|Il serre le dessin contre lui.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Nina ouvre la bouche.
+narrateur|Puis elle la referme.
+narrateur|Personne ne parle.
+narrateur|Elle observe le dessin, un instant.
+narrateur|Elle écoute la vapeur du cacao.
+papa|Tu veux le chat avec Aniss ?
+narrateur|Papa reste à la même hauteur.
+enfant-f|Papa, on fait quoi ?
+papa|On pose les mains, puis on reste.
+enfant-f|D'accord.
+narrateur|Nina reste un moment, les mains ouvertes.
+narrateur|Elle attend.
+narrateur|Aniss souffle.
+copain|Le chat bleu.
+enfant-f|J'aime le chat.
+narrateur|Aniss pose le dessin contre le plateau.
+papa|Merci, Nina.
+narrateur|Papa a vu les deux, au salon.
+maman|Le papier est tiède, sous les doigts.
+enfant-f|Il est chaud.
+narrateur|Le chat bleu tient, un peu de travers.
+enfant-f|Le chat.
+papa|Il a une oreille, là ?
+enfant-f|Oui, là.
+narrateur|Nina glisse la main près du dessin.
+narrateur|Le papier est doux, contre la peau.
+maman|Tes mains sont au chaud, Nina ?
+enfant-f|Un peu, maman.
+narrateur|Aniss s'assoit, puis se relève.
+copain|Oui.
+enfant-f|On le pose au bord ?
+maman|Le plateau va jusqu'à la table.
+enfant-f|Oui, maman.</t>
         </is>
       </c>
     </row>
@@ -1761,17 +1814,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nino croque encore une compote. Nina montre encore le chat bleu. On range les bols ? Je prends les cuillères. Le chat reste sur la table ? Oui. Il nous regarde. Tu aides à porter le bol, Nino ? Oui. Il est un peu collant. Le tapis redevient tout plat. La lune de la lampe a un peu bougé.</t>
+          <t>Ils restent près du plateau. Un verre d'eau attend près du cacao. L'eau, maintenant ! Nina pousse le verre trop vite. Une goutte penche vers le bois. Ça tombe ! Aniss ouvre la bouche. Le mot reste dedans. Dis-le, Aniss ! Aniss serre les lèvres. Nina avance les mots, trop vite. Puis elle s'arrête net. Nina referme la bouche, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le verre, un instant. Elle écoute le silence du salon. Au bord du cacao, un éclat de plateau luit. Là, sur le plateau. Tu veux le verre, Aniss ? Aniss ne dit rien. Il tend les mains, sans parler. Je veux de l'eau. Nina pousse le verre, sans se presser. Aniss le reçoit, plus lentement. Le verre est lisse et froid. Tu le vois, le verre ? Oui, papa. Le cacao est près du plateau ? Oui, maman. Aniss boit une gorgée. Nina pose une main sur la table. Le verre tient, Nina ? Oui, papa. Un rayon passe sur le plateau. Il allume le bois.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Nino croque encore une compote. Nina montre encore le chat bleu. On range les bols ? Je prends les cuillères. Le chat reste sur la table ? Oui. Il nous regarde. Tu aides à porter le bol, Nino ? Oui. Il est un peu collant. Le tapis redevient tout plat. La lune de la lampe a un peu bougé.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils restent près du plateau. Un verre d'eau attend près du cacao. L'eau, maintenant ! Nina pousse le verre trop vite. Une goutte penche vers le bois. Ça tombe ! Aniss ouvre la bouche. Le mot reste dedans. Dis-le, Aniss ! Aniss serre les lèvres. Nina avance les mots, trop vite. Puis elle s'arrête net. Nina referme la bouche, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le verre, un instant. Elle écoute le silence du salon. Au bord du cacao, un &lt;emphasis level="moderate"&gt;éclat de plateau&lt;/emphasis&gt; luit. Là, sur le plateau. Tu veux le verre, Aniss ? Aniss ne dit rien. Il tend les mains, sans parler. Je veux de l'eau. Nina pousse le verre, sans se presser. Aniss le reçoit, plus lentement. Le verre est lisse et froid. Tu le vois, le verre ? Oui, papa. Le cacao est près du plateau ? Oui, maman. Aniss boit une gorgée. Nina pose une main sur la table. Le verre tient, Nina ? Oui, papa. Un rayon passe sur le plateau. Il allume le bois.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Céleste croque une compote. Sami montre encore le chat bleu. [pause]</t>
+          <t>Ils restent près du plateau. Un verre d'eau attend près du cacao. L'eau, maintenant ! Nina pousse le verre trop vite. Une goutte penche vers le bois. Ça tombe ! Aniss ouvre la bouche. Le mot reste dedans. Dis-le, Aniss ! Aniss serre les lèvres. Nina avance les mots, trop vite. Puis elle s'arrête net. Nina referme la bouche, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le verre, un instant. Elle écoute le silence du salon. Au bord du cacao, un &lt;emphasis&gt;éclat de plateau&lt;/emphasis&gt; luit. Là, sur le plateau. Tu veux le verre, Aniss ? Aniss ne dit rien. Il tend les mains, sans parler. Je veux de l'eau. Nina pousse le verre, sans se presser. Aniss le reçoit, plus lentement. Le verre est lisse et froid. Tu le vois, le verre ? Oui, papa. Le cacao est près du plateau ? Oui, maman. Aniss boit une gorgée. Nina pose une main sur la table. Le verre tient, Nina ? Oui, papa. Un rayon passe sur le plateau. Il allume le bois. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1818,7 +1871,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1826,10 +1879,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.18</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1850,28 +1903,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de plateau</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1880,10 +1937,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1894,21 +1951,49 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=verre_trop_vite_elle_referme_la_bouche; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Nino croque encore une compote.
-narrateur|Nina montre encore le chat bleu.
-maman|On range les bols ?
-papa|Je prends les cuillères.
-enfant-m|Le chat reste sur la table ?
-maman|Oui.
-maman|Il nous regarde.
-papa|Tu aides à porter le bol, Nino ?
-enfant-m|Oui.
-enfant-m|Il est un peu collant.
-narrateur|Le tapis redevient tout plat.
-narrateur|La lune de la lampe a un peu bougé.</t>
+          <t>narrateur|Ils restent près du plateau.
+narrateur|Un verre d'eau attend près du cacao.
+enfant-f|L'eau, maintenant !
+narrateur|Nina pousse le verre trop vite.
+narrateur|Une goutte penche vers le bois.
+enfant-f|Ça tombe !
+narrateur|Aniss ouvre la bouche.
+narrateur|Le mot reste dedans.
+enfant-f|Dis-le, Aniss !
+narrateur|Aniss serre les lèvres.
+narrateur|Nina avance les mots, trop vite.
+narrateur|Puis elle s'arrête net.
+narrateur|Nina referme la bouche, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe le verre, un instant.
+narrateur|Elle écoute le silence du salon.
+narrateur|Au bord du cacao, un éclat de plateau luit.
+enfant-f|Là, sur le plateau.
+enfant-f|Tu veux le verre, Aniss ?
+narrateur|Aniss ne dit rien.
+narrateur|Il tend les mains, sans parler.
+copain|Je veux de l'eau.
+narrateur|Nina pousse le verre, sans se presser.
+narrateur|Aniss le reçoit, plus lentement.
+narrateur|Le verre est lisse et froid.
+papa|Tu le vois, le verre ?
+enfant-f|Oui, papa.
+maman|Le cacao est près du plateau ?
+enfant-f|Oui, maman.
+narrateur|Aniss boit une gorgée.
+narrateur|Nina pose une main sur la table.
+papa|Le verre tient, Nina ?
+enfant-f|Oui, papa.
+maman|Un rayon passe sur le plateau.
+enfant-f|Il allume le bois.</t>
         </is>
       </c>
     </row>
@@ -1935,17 +2020,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai attendu la fin. Bravo. Le chat bleu reste près du bol.</t>
+          <t>Ils restent près du plateau. Le chat est arrivé, Nina ? Oui, maman. Tu souffles un peu ? Oui, papa. Nina souffle, un filet d'air. Le cacao sent bon. Tu le sens, le cacao ? Oui, maman. Le dessin reste un peu, de travers. Il a tenu, sur la table. Le chat. Le plateau est chaud, sous les mains. Le chat bleu fait de l'ombre. On y retourne, après. Un éclat de plateau tient sur le bois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai attendu la fin. Bravo. Le chat bleu reste près du bol.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près du plateau. Le chat est arrivé, Nina ? Oui, maman. Tu souffles un peu ? Oui, papa. Nina souffle, un filet d'air. Le cacao sent bon. Tu le sens, le cacao ? Oui, maman. Le dessin reste un peu, de travers. Il a tenu, sur la table. Le chat. Le plateau est chaud, sous les mains. Le chat bleu fait de l'ombre. On y retourne, après. Un &lt;emphasis level="moderate"&gt;éclat de plateau&lt;/emphasis&gt; tient sur le bois.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près du plateau. Le chat est arrivé, Nina ? Oui, maman. Tu souffles un peu ? Oui, papa. Nina souffle, un filet d'air. Le cacao sent bon. Tu le sens, le cacao ? Oui, maman. Le dessin reste un peu, de travers. Il a tenu, sur la table. Le chat. Le plateau est chaud, sous les mains. Le chat bleu fait de l'ombre. On y retourne, après. Un &lt;emphasis&gt;éclat de plateau&lt;/emphasis&gt; tient sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -1992,7 +2077,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2000,10 +2085,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2012,12 +2097,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2026,17 +2111,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de plateau</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2045,11 +2134,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2058,26 +2147,43 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bois; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai attendu la fin.
-papa|Bravo.
-narrateur|Le chat bleu reste près du bol.</t>
+          <t>narrateur|Ils restent près du plateau.
+maman|Le chat est arrivé, Nina ?
+enfant-f|Oui, maman.
+papa|Tu souffles un peu ?
+enfant-f|Oui, papa.
+narrateur|Nina souffle, un filet d'air.
+enfant-f|Le cacao sent bon.
+maman|Tu le sens, le cacao ?
+enfant-f|Oui, maman.
+papa|Le dessin reste un peu, de travers.
+enfant-f|Il a tenu, sur la table.
+copain|Le chat.
+narrateur|Le plateau est chaud, sous les mains.
+narrateur|Le chat bleu fait de l'ombre.
+enfant-f|On y retourne, après.
+narrateur|Un éclat de plateau tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -2098,7 +2204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2162,6 +2268,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>